<commit_message>
Module 2 for Week-01
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04a19e4a9bb9275a/Desktop/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DA7C2B2-D27D-4A3A-85F0-552CE190A412}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41DC95B4-A2C3-4B5D-B8D7-F724A37E1F45}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,10 +94,10 @@
     <t>Account &gt; Request your data &gt; Your Orders &gt; Submit Request &gt; Download</t>
   </si>
   <si>
-    <t>Instagaram</t>
-  </si>
-  <si>
     <t>You can choose to download certain information and specify which date ranges</t>
+  </si>
+  <si>
+    <t>Instagram</t>
   </si>
 </sst>
 </file>
@@ -508,7 +508,7 @@
         <v>17</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -559,13 +559,13 @@
     </row>
     <row r="6" spans="2:8" ht="72" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2">
-        <v>45108</v>
+        <v>41456</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
@@ -577,7 +577,7 @@
         <v>17</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>